<commit_message>
refactor: unify staged transaction construction APIs
- move staged transaction, exchange, and terminal specifications into the transaction subsystem
- consolidate EventBuilder and Ledger around shared staged interfaces
- simplify event construction through staged transaction helpers
- centralize array normalization utilities
- clean up staging parameter naming for consistency
- update sample scenarios to use direct ledger construction APIs
</commit_message>
<xml_diff>
--- a/example/account-ledger.xlsx
+++ b/example/account-ledger.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Local Storage\Repositories\Finance\Lattice\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B1F8EDC-CA21-4E00-95C6-696770FF1623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E97F3838-F80A-442A-8C57-22FC9F34EBF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9555" yWindow="3015" windowWidth="18285" windowHeight="10980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51495" yWindow="3420" windowWidth="19410" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="12">
   <si>
     <t>Cash</t>
   </si>
@@ -101,12 +101,6 @@
   </si>
   <si>
     <t>Accounts Payable</t>
-  </si>
-  <si>
-    <t>Transfers to USD</t>
-  </si>
-  <si>
-    <t>Capital Gains from Disposition of A</t>
   </si>
   <si>
     <t>Transfers to B</t>
@@ -173,11 +167,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -537,21 +531,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="J1" s="2" t="s">
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="J1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
@@ -576,7 +570,7 @@
         <v>1000</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H3">
         <f>G2</f>
@@ -586,13 +580,13 @@
     </row>
     <row r="5" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C5">
         <v>500</v>
       </c>
       <c r="F5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G5">
         <v>250</v>
@@ -630,14 +624,14 @@
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D9">
         <f>C5</f>
         <v>500</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H9">
         <v>250</v>
@@ -646,7 +640,7 @@
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D10">
         <f>C8-D9</f>
@@ -687,7 +681,7 @@
     <row r="14" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
       <c r="F14" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G14">
         <f>H9</f>
@@ -695,14 +689,14 @@
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C15">
-        <v>900</v>
+        <v>800</v>
       </c>
       <c r="F15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G15">
         <v>250</v>
@@ -710,11 +704,11 @@
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C16">
         <f>SUM(D17:D18)-C15</f>
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>0</v>
@@ -723,96 +717,53 @@
         <v>500</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D17">
         <f>C12</f>
         <v>500</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D18">
         <f>C15*(G15/SUM(G14:G15))</f>
-        <v>450</v>
-      </c>
-      <c r="F18" t="s">
-        <v>0</v>
-      </c>
-      <c r="G18">
-        <f>D22/2</f>
-        <v>725</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F19" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G19">
-        <f>SUM(H20:H21)-G18</f>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C20">
-        <f>D18</f>
-        <v>450</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H20">
-        <f>G15</f>
-        <v>250</v>
-      </c>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>8</v>
-      </c>
-      <c r="C21">
-        <f>D22-C20</f>
-        <v>1000</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H21">
-        <f>G18*(C21/SUM(C20:C21))</f>
-        <v>500.00000000000006</v>
-      </c>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B22" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>1450</v>
-      </c>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F19" s="2"/>
+    </row>
+    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B20" s="2"/>
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B22" s="1"/>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" t="str" cm="1">
-        <f t="array" ref="B34:B40">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(B$2:B$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
+        <f t="array" ref="B34:B39">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(B$2:B$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
         <v>Cash</v>
       </c>
       <c r="D34" cm="1">
         <f t="array" ref="D34">SUMPRODUCT(--(B34=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>0</v>
+        <v>1350</v>
       </c>
       <c r="F34" t="str" cm="1">
-        <f t="array" ref="F34:F38">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(F$2:F$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
+        <f t="array" ref="F34:F37">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(F$2:F$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
         <v>Cash</v>
       </c>
       <c r="H34" cm="1">
         <f t="array" ref="H34">SUMPRODUCT(--(F34=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>725</v>
+        <v>0</v>
       </c>
       <c r="J34" t="e" cm="1" vm="1">
         <f t="array" ref="J34">_xlfn.LET(_xlpm.x,_xlfn.UNIQUE(J$2:J$33),_xlfn._xlws.FILTER(_xlpm.x,_xlpm.x&lt;&gt;0))</f>
@@ -836,7 +787,7 @@
       </c>
       <c r="H35" cm="1">
         <f t="array" ref="H35">SUMPRODUCT(--(F35=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>-500.00000000000006</v>
+        <v>0</v>
       </c>
       <c r="L35" cm="1">
         <f t="array" ref="L35">SUMPRODUCT(--(J35=J$2:J$33),K$2:K$33-L$2:L$33)</f>
@@ -849,7 +800,7 @@
       </c>
       <c r="D36" cm="1">
         <f t="array" ref="D36">SUMPRODUCT(--(B36=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="F36" t="str">
         <v>Accounts Payable</v>
@@ -876,7 +827,7 @@
       </c>
       <c r="H37" cm="1">
         <f t="array" ref="H37">SUMPRODUCT(--(F37=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="L37" cm="1">
         <f t="array" ref="L37">SUMPRODUCT(--(J37=J$2:J$33),K$2:K$33-L$2:L$33)</f>
@@ -885,18 +836,15 @@
     </row>
     <row r="38" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" t="str">
-        <v>Transfers to USD</v>
+        <v>Capital Loss from Disposition of B</v>
       </c>
       <c r="D38" cm="1">
         <f t="array" ref="D38">SUMPRODUCT(--(B38=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>500</v>
-      </c>
-      <c r="F38" t="str">
-        <v>Capital Gains from Disposition of A</v>
+        <v>100</v>
       </c>
       <c r="H38" cm="1">
         <f t="array" ref="H38">SUMPRODUCT(--(F38=F$2:F$33),G$2:G$33-H$2:H$33)</f>
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="L38" cm="1">
         <f t="array" ref="L38">SUMPRODUCT(--(J38=J$2:J$33),K$2:K$33-L$2:L$33)</f>
@@ -905,11 +853,11 @@
     </row>
     <row r="39" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" t="str">
-        <v>Capital Loss from Disposition of B</v>
+        <v>Transfers from B</v>
       </c>
       <c r="D39" cm="1">
         <f t="array" ref="D39">SUMPRODUCT(--(B39=B$2:B$33),C$2:C$33-D$2:D$33)</f>
-        <v>50</v>
+        <v>-400</v>
       </c>
       <c r="H39" cm="1">
         <f t="array" ref="H39">SUMPRODUCT(--(F39=F$2:F$33),G$2:G$33-H$2:H$33)</f>
@@ -921,9 +869,6 @@
       </c>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B40" t="str">
-        <v>Transfers from B</v>
-      </c>
       <c r="D40" cm="1">
         <f t="array" ref="D40">SUMPRODUCT(--(B40=B$2:B$33),C$2:C$33-D$2:D$33)</f>
         <v>0</v>

</xml_diff>